<commit_message>
Fix camera glitches, swap export reports logic, and improve UI
</commit_message>
<xml_diff>
--- a/Attendance/Cricket/attendance_report.xlsx
+++ b/Attendance/Cricket/attendance_report.xlsx
@@ -471,12 +471,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Karan</t>
+          <t>Dhruv</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -491,7 +491,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -501,12 +501,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>⚠ Low</t>
+          <t>✅ Good</t>
         </is>
       </c>
     </row>

</xml_diff>